<commit_message>
Code updates DeleteColumns and DeleteRows
</commit_message>
<xml_diff>
--- a/Autossential.Workbook.Activities.Tests/Assets/Data.xlsx
+++ b/Autossential.Workbook.Activities.Tests/Assets/Data.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="SparseRows" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t xml:space="preserve">a</t>
   </si>
@@ -52,16 +52,10 @@
     <t xml:space="preserve">q</t>
   </si>
   <si>
-    <t xml:space="preserve">c</t>
-  </si>
-  <si>
     <t xml:space="preserve">e</t>
   </si>
   <si>
     <t xml:space="preserve">g</t>
-  </si>
-  <si>
-    <t xml:space="preserve">h</t>
   </si>
 </sst>
 </file>
@@ -439,7 +433,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="17.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="4" width="7.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16374" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16374" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -638,7 +632,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -648,29 +642,26 @@
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="H1" s="7"/>
+      <c r="I1" s="0" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B1:D1"/>
-    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="G1:H1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>